<commit_message>
Add tight Skagway downtown narration redo
</commit_message>
<xml_diff>
--- a/transcripts/Time_point_Skagway_Downtown.xlsx
+++ b/transcripts/Time_point_Skagway_Downtown.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xieyulong2022/AI_Learn/Codex/voice_clone_NextStage/transcripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5725173-BE6B-DC47-B08C-0D69FEB0888A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41FDF2CE-E86B-4441-B280-98829A5A1F43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1980" yWindow="2600" windowWidth="26440" windowHeight="14660" activeTab="1" xr2:uid="{4EBE08BA-59A5-4A4A-9488-F78565F80119}"/>
+    <workbookView xWindow="740" yWindow="600" windowWidth="26460" windowHeight="14680" activeTab="2" xr2:uid="{4EBE08BA-59A5-4A4A-9488-F78565F80119}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="109">
   <si>
     <t>alaska_cruise_2026,SD001,001,00:00:00,00:00:12,"来到史凯威，最先映入眼帘的，就是这座淘金者纪念雕像。","Arriving in Skagway, the first thing we see is this Gold Rush monument.",Gold Rush Monument.,reviewed</t>
   </si>
@@ -518,6 +519,51 @@
   </si>
   <si>
     <t>在以商店和酒馆闻名的淘金小镇里，也保存着</t>
+  </si>
+  <si>
+    <t>今天是我们乘坐 公主邮轮的发现号从加拿大温哥华出发后的第五天，我们来到了阿拉斯加的史凯威。</t>
+  </si>
+  <si>
+    <t>另外三艘邮轮也陆续抵达了 史凯威。我们的 公主邮轮的发现号今天没有直接靠岸，需要乘接驳船上岸。这与几年前港口发生的山体滑坡以及码头安全限制有关。</t>
+  </si>
+  <si>
+    <t>这里是历史悠久的 白隘口火车站。</t>
+  </si>
+  <si>
+    <t>这台巨大的机器是 白隘口铁路使用过的旋转式除雪车，前方的巨大叶轮专门用来清除山间铁路上的厚雪。</t>
+  </si>
+  <si>
+    <t>从这里开始，我们沿着 史凯威 最著名的 百老汇大街慢慢往前走。</t>
+  </si>
+  <si>
+    <t>前面带有金色圆顶的是 史凯威 著名的 黄金北方酒店，也是 百老汇上很容易辨认的历史建筑。</t>
+  </si>
+  <si>
+    <t>这座外墙非常特别的建筑就是当年的“北极兄弟会会馆”，它的外墙全部由漂流木拼接而成。</t>
+  </si>
+  <si>
+    <t>万神殿曾是淘金热时期最豪华的剧院之一，也是当年歌舞表演的重要场所。</t>
+  </si>
+  <si>
+    <t>前面这座很醒目的石头建筑是史凯威市政厅.  它最初计划作为一所学校使用。  它也是史凯威唯一的石砌建筑，</t>
+  </si>
+  <si>
+    <t>这里是历史悠久的 柯姆斯奇珍店。</t>
+  </si>
+  <si>
+    <t>这栋黄绿相间的建筑是历史上的林奇与肯尼迪男装及百货商店</t>
+  </si>
+  <si>
+    <t>来到史凯威,我们当然也没有错过这里很有名的克朗代克炸面饼店,刚出炉的 油炸面饼外酥内软,再撒上一层肉桂糖和糖粉，香气扑鼻。,虽然只是简单的一块炸面团，却成为许多游客来到史凯威最难忘的味道。我们也买了一些，趁热尝尝。</t>
+  </si>
+  <si>
+    <t>逛完 史凯威市中心，我们沿着原路慢慢返回港口。</t>
+  </si>
+  <si>
+    <t>这是我们第二次来到 史凯威。和上一次一样，这座小城给我的感觉并不只是一个邮轮港口。短短几条街上仍然保存着许多克朗代克淘金热留下来的建筑和故事。上午的市区漫步也只是今天行程的前半段。接下来，我们将回到港口，登上白隘口景观列车。沿着一百多年前淘金者走过的方向进入群山，开始今天下午最精彩的一段旅程</t>
+  </si>
+  <si>
+    <t>11:45;15</t>
   </si>
 </sst>
 </file>
@@ -573,13 +619,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="21" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1639,4 +1686,206 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D056E81-B8F5-D744-B6A9-B76511F6D85F}">
+  <dimension ref="A1:B33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="5">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="5">
+        <v>5.4884259259259258E-2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="5">
+        <v>0.18425925925925926</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="5">
+        <v>0.20296296296296296</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>0.21339120370370371</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>0.2326388888888889</v>
+      </c>
+      <c r="B7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>0.26412037037037039</v>
+      </c>
+      <c r="B8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>0.29046296296296298</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <v>0.3472337962962963</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>0.37247685185185186</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <v>0.37853009259259257</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>0.38630787037037034</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="5">
+        <v>0.48163194444444446</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="5"/>
+      <c r="B16" s="4"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="5"/>
+      <c r="B17" s="4"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="5"/>
+      <c r="B18" s="4"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="5"/>
+      <c r="B19" s="4"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="5"/>
+      <c r="B20" s="4"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="5"/>
+      <c r="B21" s="4"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="5"/>
+      <c r="B22" s="4"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="5"/>
+      <c r="B23" s="4"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="5"/>
+      <c r="B24" s="4"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="5"/>
+      <c r="B25" s="4"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="5"/>
+      <c r="B26" s="4"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="5"/>
+      <c r="B27" s="4"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="5"/>
+      <c r="B28" s="4"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="5"/>
+      <c r="B29" s="4"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="5"/>
+      <c r="B30" s="4"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="5"/>
+      <c r="B31" s="4"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="5"/>
+      <c r="B32" s="4"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="5"/>
+      <c r="B33" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>